<commit_message>
補兆豐 2020-2021 期數(OCI);AC/Trading 該期兆豐無部位
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/銀行債券_完整報表.xlsx
+++ b/銀行債券_完整報表.xlsx
@@ -9738,7 +9738,9 @@
       <c r="B3" s="4" t="n">
         <v>1316</v>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D3" s="4" t="n">
         <v>0</v>
       </c>
@@ -9751,7 +9753,9 @@
       <c r="G3" s="4" t="n">
         <v>1206</v>
       </c>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" s="4" t="n">
         <v>1957</v>
       </c>
@@ -9764,7 +9768,9 @@
       <c r="L3" s="4" t="n">
         <v>902</v>
       </c>
-      <c r="M3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N3" s="4" t="n">
         <v>1817</v>
       </c>
@@ -9777,7 +9783,9 @@
       <c r="Q3" s="4" t="n">
         <v>1231</v>
       </c>
-      <c r="R3" s="4" t="inlineStr"/>
+      <c r="R3" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S3" s="4" t="n">
         <v>1684</v>
       </c>
@@ -9927,7 +9935,9 @@
       <c r="B4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D4" s="4" t="n">
         <v>0</v>
       </c>
@@ -9940,7 +9950,9 @@
       <c r="G4" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" s="4" t="n">
         <v>355</v>
       </c>
@@ -9953,7 +9965,9 @@
       <c r="L4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="M4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N4" s="4" t="n">
         <v>239</v>
       </c>
@@ -9966,7 +9980,9 @@
       <c r="Q4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="R4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S4" s="4" t="n">
         <v>174</v>
       </c>
@@ -10116,7 +10132,9 @@
       <c r="B5" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D5" s="4" t="n">
         <v>0</v>
       </c>
@@ -10129,7 +10147,9 @@
       <c r="G5" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" s="4" t="n">
         <v>63</v>
       </c>
@@ -10142,7 +10162,9 @@
       <c r="L5" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N5" s="4" t="n">
         <v>136</v>
       </c>
@@ -10155,7 +10177,9 @@
       <c r="Q5" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="R5" s="4" t="inlineStr"/>
+      <c r="R5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S5" s="4" t="n">
         <v>188</v>
       </c>
@@ -10305,7 +10329,9 @@
       <c r="B6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D6" s="4" t="n">
         <v>0</v>
       </c>
@@ -10318,7 +10344,9 @@
       <c r="G6" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" s="4" t="n">
         <v>84</v>
       </c>
@@ -10331,7 +10359,9 @@
       <c r="L6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N6" s="4" t="n">
         <v>234</v>
       </c>
@@ -10344,7 +10374,9 @@
       <c r="Q6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S6" s="4" t="n">
         <v>369</v>
       </c>
@@ -10494,7 +10526,9 @@
       <c r="B7" s="4" t="n">
         <v>445</v>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="n">
+        <v>501</v>
+      </c>
       <c r="D7" s="4" t="n">
         <v>0</v>
       </c>
@@ -10507,7 +10541,9 @@
       <c r="G7" s="4" t="n">
         <v>541</v>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="n">
+        <v>364</v>
+      </c>
       <c r="I7" s="4" t="n">
         <v>709</v>
       </c>
@@ -10520,7 +10556,9 @@
       <c r="L7" s="4" t="n">
         <v>367</v>
       </c>
-      <c r="M7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="n">
+        <v>402</v>
+      </c>
       <c r="N7" s="4" t="n">
         <v>416</v>
       </c>
@@ -10533,7 +10571,9 @@
       <c r="Q7" s="4" t="n">
         <v>330</v>
       </c>
-      <c r="R7" s="4" t="inlineStr"/>
+      <c r="R7" s="4" t="n">
+        <v>498</v>
+      </c>
       <c r="S7" s="4" t="n">
         <v>368</v>
       </c>
@@ -10683,7 +10723,9 @@
       <c r="B8" s="4" t="n">
         <v>101</v>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="n">
+        <v>962</v>
+      </c>
       <c r="D8" s="4" t="n">
         <v>0</v>
       </c>
@@ -10696,7 +10738,9 @@
       <c r="G8" s="4" t="n">
         <v>176</v>
       </c>
-      <c r="H8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="n">
+        <v>1024</v>
+      </c>
       <c r="I8" s="4" t="n">
         <v>947</v>
       </c>
@@ -10709,7 +10753,9 @@
       <c r="L8" s="4" t="n">
         <v>149</v>
       </c>
-      <c r="M8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="n">
+        <v>1045</v>
+      </c>
       <c r="N8" s="4" t="n">
         <v>1120</v>
       </c>
@@ -10722,7 +10768,9 @@
       <c r="Q8" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="R8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="n">
+        <v>1053</v>
+      </c>
       <c r="S8" s="4" t="n">
         <v>134</v>
       </c>
@@ -10872,7 +10920,9 @@
       <c r="B9" s="4" t="n">
         <v>1445</v>
       </c>
-      <c r="C9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="D9" s="4" t="n">
         <v>0</v>
       </c>
@@ -10885,7 +10935,9 @@
       <c r="G9" s="4" t="n">
         <v>1485</v>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="n">
+        <v>9</v>
+      </c>
       <c r="I9" s="4" t="n">
         <v>626</v>
       </c>
@@ -10898,7 +10950,9 @@
       <c r="L9" s="4" t="n">
         <v>1132</v>
       </c>
-      <c r="M9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="n">
+        <v>11</v>
+      </c>
       <c r="N9" s="4" t="n">
         <v>593</v>
       </c>
@@ -10911,7 +10965,9 @@
       <c r="Q9" s="4" t="n">
         <v>1080</v>
       </c>
-      <c r="R9" s="4" t="inlineStr"/>
+      <c r="R9" s="4" t="n">
+        <v>8</v>
+      </c>
       <c r="S9" s="4" t="n">
         <v>168</v>
       </c>
@@ -11061,7 +11117,9 @@
       <c r="B10" s="4" t="n">
         <v>1822</v>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D10" s="4" t="n">
         <v>0</v>
       </c>
@@ -11074,7 +11132,9 @@
       <c r="G10" s="4" t="n">
         <v>1803</v>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="4" t="n">
         <v>96</v>
       </c>
@@ -11087,7 +11147,9 @@
       <c r="L10" s="4" t="n">
         <v>1902</v>
       </c>
-      <c r="M10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N10" s="4" t="n">
         <v>288</v>
       </c>
@@ -11100,7 +11162,9 @@
       <c r="Q10" s="4" t="n">
         <v>2088</v>
       </c>
-      <c r="R10" s="4" t="inlineStr"/>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S10" s="4" t="n">
         <v>377</v>
       </c>
@@ -11250,7 +11314,9 @@
       <c r="B11" s="4" t="n">
         <v>586</v>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D11" s="4" t="n">
         <v>0</v>
       </c>
@@ -11263,7 +11329,9 @@
       <c r="G11" s="4" t="n">
         <v>571</v>
       </c>
-      <c r="H11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I11" s="4" t="n">
         <v>123</v>
       </c>
@@ -11276,7 +11344,9 @@
       <c r="L11" s="4" t="n">
         <v>665</v>
       </c>
-      <c r="M11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N11" s="4" t="n">
         <v>137</v>
       </c>
@@ -11289,7 +11359,9 @@
       <c r="Q11" s="4" t="n">
         <v>657</v>
       </c>
-      <c r="R11" s="4" t="inlineStr"/>
+      <c r="R11" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S11" s="4" t="n">
         <v>135</v>
       </c>
@@ -11439,7 +11511,9 @@
       <c r="B12" s="4" t="n">
         <v>162</v>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D12" s="4" t="n">
         <v>0</v>
       </c>
@@ -11452,7 +11526,9 @@
       <c r="G12" s="4" t="n">
         <v>175</v>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I12" s="4" t="n">
         <v>106</v>
       </c>
@@ -11465,7 +11541,9 @@
       <c r="L12" s="4" t="n">
         <v>267</v>
       </c>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="N12" s="4" t="n">
         <v>178</v>
       </c>
@@ -11478,7 +11556,9 @@
       <c r="Q12" s="4" t="n">
         <v>259</v>
       </c>
-      <c r="R12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="S12" s="4" t="n">
         <v>171</v>
       </c>

</xml_diff>